<commit_message>
Backup: push all files before cleaning
</commit_message>
<xml_diff>
--- a/data/raw/data_sorted.xlsx
+++ b/data/raw/data_sorted.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Morta\OneDrive\Desktop\Gam3a\MARS\Integrated Project\data\raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A65ED3C1-093A-4549-8C5D-40DE4FA0DC3E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B16B84C4-D03C-47C9-A70A-82EEF83E7646}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="6" xr2:uid="{E0559C20-5939-423D-BFBD-814363ADABA6}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="11">
   <si>
     <t>C:\Users\Morta\OneDrive\Desktop\Gam3a\MARS\Integrated Project\data\raw\essai donnees paye.xlsx</t>
   </si>
@@ -75,9 +75,6 @@
   </si>
   <si>
     <t>TOTAL</t>
-  </si>
-  <si>
-    <t>test</t>
   </si>
 </sst>
 </file>
@@ -486,14 +483,14 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E3C40221-1FB8-4E4C-845C-D82F7D9B3102}">
-  <dimension ref="A1:J20"/>
+  <dimension ref="A1:I20"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14.77734375" customWidth="1"/>
-    <col min="2" max="10" width="18.77734375" customWidth="1"/>
+    <col min="2" max="9" width="18.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
@@ -521,216 +518,441 @@
       <c r="I1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="J1" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>14</v>
       </c>
       <c r="B2" s="2">
         <v>2800</v>
       </c>
-      <c r="J2" s="2">
-        <v>2800</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C2" s="2">
+        <v>1159.49</v>
+      </c>
+      <c r="D2" s="2">
+        <v>462.09000000000015</v>
+      </c>
+      <c r="E2" s="2">
+        <v>-2000.03</v>
+      </c>
+      <c r="G2" s="2">
+        <v>2000.03</v>
+      </c>
+      <c r="I2" s="2">
+        <v>3262.09</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>16</v>
       </c>
       <c r="B3" s="2">
         <v>3000</v>
       </c>
-      <c r="J3" s="2">
-        <v>3000</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C3" s="2">
+        <v>1069.79</v>
+      </c>
+      <c r="D3" s="2">
+        <v>446.46000000000004</v>
+      </c>
+      <c r="E3" s="2">
+        <v>-2231.77</v>
+      </c>
+      <c r="G3" s="2">
+        <v>2231.77</v>
+      </c>
+      <c r="I3" s="2">
+        <v>3446.46</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>11</v>
       </c>
       <c r="B4" s="2">
         <v>2802.59</v>
       </c>
-      <c r="J4" s="2">
-        <v>2802.59</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C4" s="2">
+        <v>1160.3600000000001</v>
+      </c>
+      <c r="D4" s="2">
+        <v>462.42000000000007</v>
+      </c>
+      <c r="E4" s="2">
+        <v>-2020.23</v>
+      </c>
+      <c r="G4" s="2">
+        <v>2020.23</v>
+      </c>
+      <c r="I4" s="2">
+        <v>3265.01</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>3</v>
       </c>
       <c r="B5" s="2">
         <v>3678.62</v>
       </c>
-      <c r="J5" s="2">
-        <v>3678.62</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C5" s="2">
+        <v>1311.78</v>
+      </c>
+      <c r="D5" s="2">
+        <v>545.68000000000029</v>
+      </c>
+      <c r="E5" s="2">
+        <v>-2795.07</v>
+      </c>
+      <c r="G5" s="2">
+        <v>2795.07</v>
+      </c>
+      <c r="I5" s="2">
+        <v>4224.3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>4</v>
       </c>
       <c r="B6" s="2">
         <v>22326.61</v>
       </c>
-      <c r="J6" s="2">
-        <v>22326.61</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C6" s="2">
+        <v>11684.61</v>
+      </c>
+      <c r="D6" s="2">
+        <v>6829.68</v>
+      </c>
+      <c r="E6" s="2">
+        <v>-14066.69</v>
+      </c>
+      <c r="G6" s="2">
+        <v>14066.69</v>
+      </c>
+      <c r="I6" s="2">
+        <v>29156.29</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>13</v>
       </c>
       <c r="B7" s="2">
         <v>3105.75</v>
       </c>
-      <c r="J7" s="2">
-        <v>3105.75</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C7" s="2">
+        <v>1107.51</v>
+      </c>
+      <c r="D7" s="2">
+        <v>461.92000000000007</v>
+      </c>
+      <c r="E7" s="2">
+        <v>-2297.44</v>
+      </c>
+      <c r="G7" s="2">
+        <v>2297.44</v>
+      </c>
+      <c r="I7" s="2">
+        <v>3567.67</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>17</v>
       </c>
       <c r="B8" s="2">
         <v>5417</v>
       </c>
-      <c r="J8" s="2">
-        <v>5417</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C8" s="2">
+        <v>3604.8399999999997</v>
+      </c>
+      <c r="D8" s="2">
+        <v>2371.1899999999996</v>
+      </c>
+      <c r="E8" s="2">
+        <v>-4090.55</v>
+      </c>
+      <c r="G8" s="2">
+        <v>4090.55</v>
+      </c>
+      <c r="I8" s="2">
+        <v>7788.19</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>6</v>
       </c>
       <c r="B9" s="2">
         <v>3381</v>
       </c>
-      <c r="J9" s="2">
-        <v>3381</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C9" s="2">
+        <v>1205.6500000000001</v>
+      </c>
+      <c r="D9" s="2">
+        <v>504.76000000000022</v>
+      </c>
+      <c r="E9" s="2">
+        <v>-2558.33</v>
+      </c>
+      <c r="G9" s="2">
+        <v>2558.33</v>
+      </c>
+      <c r="I9" s="2">
+        <v>3885.76</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>15</v>
       </c>
       <c r="B10" s="2">
         <v>3201.06</v>
       </c>
-      <c r="J10" s="2">
-        <v>3201.06</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C10" s="2">
+        <v>1338.59</v>
+      </c>
+      <c r="D10" s="2">
+        <v>562.05000000000018</v>
+      </c>
+      <c r="E10" s="2">
+        <v>-2338.25</v>
+      </c>
+      <c r="G10" s="2">
+        <v>2338.25</v>
+      </c>
+      <c r="I10" s="2">
+        <v>3763.11</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>5</v>
       </c>
       <c r="B11" s="2">
         <v>3312.22</v>
       </c>
-      <c r="J11" s="2">
-        <v>3312.22</v>
-      </c>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C11" s="2">
+        <v>1138.42</v>
+      </c>
+      <c r="D11" s="2">
+        <v>435.43000000000029</v>
+      </c>
+      <c r="E11" s="2">
+        <v>-2474.0300000000002</v>
+      </c>
+      <c r="G11" s="2">
+        <v>2474.0300000000002</v>
+      </c>
+      <c r="I11" s="2">
+        <v>3747.65</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>7</v>
       </c>
       <c r="B12" s="2">
         <v>3531</v>
       </c>
-      <c r="J12" s="2">
-        <v>3531</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C12" s="2">
+        <v>1259.1399999999999</v>
+      </c>
+      <c r="D12" s="2">
+        <v>599.0600000000004</v>
+      </c>
+      <c r="E12" s="2">
+        <v>-2521.16</v>
+      </c>
+      <c r="G12" s="2">
+        <v>2521.16</v>
+      </c>
+      <c r="I12" s="2">
+        <v>4130.0600000000004</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>12</v>
       </c>
       <c r="B13" s="2">
         <v>2805.19</v>
       </c>
-      <c r="J13" s="2">
-        <v>2805.19</v>
-      </c>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C13" s="2">
+        <v>1161.27</v>
+      </c>
+      <c r="D13" s="2">
+        <v>462.77999999999975</v>
+      </c>
+      <c r="E13" s="2">
+        <v>-1974.25</v>
+      </c>
+      <c r="G13" s="2">
+        <v>1974.25</v>
+      </c>
+      <c r="I13" s="2">
+        <v>3267.97</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>18</v>
       </c>
       <c r="B14" s="2">
         <v>3903.3</v>
       </c>
-      <c r="J14" s="2">
-        <v>3903.3</v>
-      </c>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C14" s="2">
+        <v>1391.9099999999999</v>
+      </c>
+      <c r="D14" s="2">
+        <v>575.9399999999996</v>
+      </c>
+      <c r="E14" s="2">
+        <v>-3087.33</v>
+      </c>
+      <c r="G14" s="2">
+        <v>3087.33</v>
+      </c>
+      <c r="I14" s="2">
+        <v>4479.24</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>1</v>
       </c>
       <c r="B15" s="2">
         <v>5247.83</v>
       </c>
-      <c r="J15" s="2">
-        <v>5247.83</v>
-      </c>
-    </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C15" s="2">
+        <v>2194.1</v>
+      </c>
+      <c r="D15" s="2">
+        <v>978.25</v>
+      </c>
+      <c r="E15" s="2">
+        <v>-3723.76</v>
+      </c>
+      <c r="G15" s="2">
+        <v>3723.76</v>
+      </c>
+      <c r="I15" s="2">
+        <v>6226.08</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>9</v>
       </c>
       <c r="B16" s="2">
         <v>2702.51</v>
       </c>
-      <c r="J16" s="2">
-        <v>2702.51</v>
-      </c>
-    </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C16" s="2">
+        <v>1125.96</v>
+      </c>
+      <c r="D16" s="2">
+        <v>449.25999999999976</v>
+      </c>
+      <c r="E16" s="2">
+        <v>-2025.81</v>
+      </c>
+      <c r="G16" s="2">
+        <v>2025.81</v>
+      </c>
+      <c r="I16" s="2">
+        <v>3151.77</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>2</v>
       </c>
       <c r="B17" s="2">
         <v>5533.46</v>
       </c>
-      <c r="J17" s="2">
-        <v>5533.46</v>
-      </c>
-    </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C17" s="2">
+        <v>2320.1099999999997</v>
+      </c>
+      <c r="D17" s="2">
+        <v>1066.8900000000003</v>
+      </c>
+      <c r="E17" s="2">
+        <v>-3661.84</v>
+      </c>
+      <c r="G17" s="2">
+        <v>3661.84</v>
+      </c>
+      <c r="I17" s="2">
+        <v>6600.35</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>20</v>
       </c>
       <c r="B18" s="2">
         <v>6747.71</v>
       </c>
-      <c r="J18" s="2">
-        <v>6747.71</v>
-      </c>
-    </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C18" s="2">
+        <v>4603.0600000000004</v>
+      </c>
+      <c r="D18" s="2">
+        <v>3096.6500000000005</v>
+      </c>
+      <c r="E18" s="2">
+        <v>-4657.79</v>
+      </c>
+      <c r="G18" s="2">
+        <v>4657.79</v>
+      </c>
+      <c r="I18" s="2">
+        <v>9844.36</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>19</v>
       </c>
       <c r="B19" s="2">
         <v>4250</v>
       </c>
-      <c r="J19" s="2">
-        <v>4250</v>
-      </c>
-    </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C19" s="2">
+        <v>1753.94</v>
+      </c>
+      <c r="D19" s="2">
+        <v>753.01000000000022</v>
+      </c>
+      <c r="E19" s="2">
+        <v>-2905.89</v>
+      </c>
+      <c r="G19" s="2">
+        <v>2905.89</v>
+      </c>
+      <c r="I19" s="2">
+        <v>5003.01</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>10</v>
       </c>
       <c r="B20" s="2">
         <v>0</v>
       </c>
-      <c r="J20" s="2">
+      <c r="C20" s="2">
+        <v>0</v>
+      </c>
+      <c r="D20" s="2">
+        <v>0</v>
+      </c>
+      <c r="E20" s="2">
+        <v>0</v>
+      </c>
+      <c r="G20" s="2">
+        <v>0</v>
+      </c>
+      <c r="I20" s="2">
         <v>0</v>
       </c>
     </row>
@@ -741,14 +963,14 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{47A78E01-326D-40F2-A036-CB85B51465D1}">
-  <dimension ref="A1:J20"/>
+  <dimension ref="A1:I20"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14.77734375" customWidth="1"/>
-    <col min="2" max="10" width="18.77734375" customWidth="1"/>
+    <col min="2" max="9" width="18.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
@@ -776,216 +998,441 @@
       <c r="I1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="J1" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>14</v>
       </c>
       <c r="B2" s="2">
         <v>2800</v>
       </c>
-      <c r="J2" s="2">
-        <v>2800</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C2" s="2">
+        <v>1159.49</v>
+      </c>
+      <c r="D2" s="2">
+        <v>462.09000000000015</v>
+      </c>
+      <c r="E2" s="2">
+        <v>-2000.03</v>
+      </c>
+      <c r="G2" s="2">
+        <v>2000.03</v>
+      </c>
+      <c r="I2" s="2">
+        <v>3262.09</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>16</v>
       </c>
       <c r="B3" s="2">
         <v>3000</v>
       </c>
-      <c r="J3" s="2">
-        <v>3000</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C3" s="2">
+        <v>1069.79</v>
+      </c>
+      <c r="D3" s="2">
+        <v>446.46000000000004</v>
+      </c>
+      <c r="E3" s="2">
+        <v>-2231.77</v>
+      </c>
+      <c r="G3" s="2">
+        <v>2231.77</v>
+      </c>
+      <c r="I3" s="2">
+        <v>3446.46</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>11</v>
       </c>
       <c r="B4" s="2">
         <v>2802.59</v>
       </c>
-      <c r="J4" s="2">
-        <v>2802.59</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C4" s="2">
+        <v>1160.3600000000001</v>
+      </c>
+      <c r="D4" s="2">
+        <v>462.42000000000007</v>
+      </c>
+      <c r="E4" s="2">
+        <v>-2020.23</v>
+      </c>
+      <c r="G4" s="2">
+        <v>2020.23</v>
+      </c>
+      <c r="I4" s="2">
+        <v>3265.01</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>3</v>
       </c>
       <c r="B5" s="2">
         <v>3678.62</v>
       </c>
-      <c r="J5" s="2">
-        <v>3678.62</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C5" s="2">
+        <v>1311.78</v>
+      </c>
+      <c r="D5" s="2">
+        <v>545.68000000000029</v>
+      </c>
+      <c r="E5" s="2">
+        <v>-2795.07</v>
+      </c>
+      <c r="G5" s="2">
+        <v>2795.07</v>
+      </c>
+      <c r="I5" s="2">
+        <v>4224.3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>4</v>
       </c>
       <c r="B6" s="2">
         <v>22326.61</v>
       </c>
-      <c r="J6" s="2">
-        <v>22326.61</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C6" s="2">
+        <v>11684.61</v>
+      </c>
+      <c r="D6" s="2">
+        <v>6829.68</v>
+      </c>
+      <c r="E6" s="2">
+        <v>-14066.69</v>
+      </c>
+      <c r="G6" s="2">
+        <v>14066.69</v>
+      </c>
+      <c r="I6" s="2">
+        <v>29156.29</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>13</v>
       </c>
       <c r="B7" s="2">
         <v>3105.75</v>
       </c>
-      <c r="J7" s="2">
-        <v>3105.75</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C7" s="2">
+        <v>1107.51</v>
+      </c>
+      <c r="D7" s="2">
+        <v>461.92000000000007</v>
+      </c>
+      <c r="E7" s="2">
+        <v>-2297.44</v>
+      </c>
+      <c r="G7" s="2">
+        <v>2297.44</v>
+      </c>
+      <c r="I7" s="2">
+        <v>3567.67</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>17</v>
       </c>
       <c r="B8" s="2">
         <v>5417</v>
       </c>
-      <c r="J8" s="2">
-        <v>5417</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C8" s="2">
+        <v>3604.8399999999997</v>
+      </c>
+      <c r="D8" s="2">
+        <v>2371.1899999999996</v>
+      </c>
+      <c r="E8" s="2">
+        <v>-4090.55</v>
+      </c>
+      <c r="G8" s="2">
+        <v>4090.55</v>
+      </c>
+      <c r="I8" s="2">
+        <v>7788.19</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>6</v>
       </c>
       <c r="B9" s="2">
         <v>3381</v>
       </c>
-      <c r="J9" s="2">
-        <v>3381</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C9" s="2">
+        <v>1205.6500000000001</v>
+      </c>
+      <c r="D9" s="2">
+        <v>504.76000000000022</v>
+      </c>
+      <c r="E9" s="2">
+        <v>-2558.33</v>
+      </c>
+      <c r="G9" s="2">
+        <v>2558.33</v>
+      </c>
+      <c r="I9" s="2">
+        <v>3885.76</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>15</v>
       </c>
       <c r="B10" s="2">
         <v>3201.06</v>
       </c>
-      <c r="J10" s="2">
-        <v>3201.06</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C10" s="2">
+        <v>1338.59</v>
+      </c>
+      <c r="D10" s="2">
+        <v>562.05000000000018</v>
+      </c>
+      <c r="E10" s="2">
+        <v>-2338.25</v>
+      </c>
+      <c r="G10" s="2">
+        <v>2338.25</v>
+      </c>
+      <c r="I10" s="2">
+        <v>3763.11</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>5</v>
       </c>
       <c r="B11" s="2">
         <v>3312.22</v>
       </c>
-      <c r="J11" s="2">
-        <v>3312.22</v>
-      </c>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C11" s="2">
+        <v>1138.42</v>
+      </c>
+      <c r="D11" s="2">
+        <v>435.43000000000029</v>
+      </c>
+      <c r="E11" s="2">
+        <v>-2474.0300000000002</v>
+      </c>
+      <c r="G11" s="2">
+        <v>2474.0300000000002</v>
+      </c>
+      <c r="I11" s="2">
+        <v>3747.65</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>7</v>
       </c>
       <c r="B12" s="2">
         <v>3531</v>
       </c>
-      <c r="J12" s="2">
-        <v>3531</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C12" s="2">
+        <v>1259.1399999999999</v>
+      </c>
+      <c r="D12" s="2">
+        <v>599.0600000000004</v>
+      </c>
+      <c r="E12" s="2">
+        <v>-2521.16</v>
+      </c>
+      <c r="G12" s="2">
+        <v>2521.16</v>
+      </c>
+      <c r="I12" s="2">
+        <v>4130.0600000000004</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>12</v>
       </c>
       <c r="B13" s="2">
         <v>2805.19</v>
       </c>
-      <c r="J13" s="2">
-        <v>2805.19</v>
-      </c>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C13" s="2">
+        <v>1161.27</v>
+      </c>
+      <c r="D13" s="2">
+        <v>462.77999999999975</v>
+      </c>
+      <c r="E13" s="2">
+        <v>-1974.25</v>
+      </c>
+      <c r="G13" s="2">
+        <v>1974.25</v>
+      </c>
+      <c r="I13" s="2">
+        <v>3267.97</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>18</v>
       </c>
       <c r="B14" s="2">
         <v>3903.3</v>
       </c>
-      <c r="J14" s="2">
-        <v>3903.3</v>
-      </c>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C14" s="2">
+        <v>1391.9099999999999</v>
+      </c>
+      <c r="D14" s="2">
+        <v>575.9399999999996</v>
+      </c>
+      <c r="E14" s="2">
+        <v>-3087.33</v>
+      </c>
+      <c r="G14" s="2">
+        <v>3087.33</v>
+      </c>
+      <c r="I14" s="2">
+        <v>4479.24</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>1</v>
       </c>
       <c r="B15" s="2">
         <v>5247.83</v>
       </c>
-      <c r="J15" s="2">
-        <v>5247.83</v>
-      </c>
-    </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C15" s="2">
+        <v>2194.1</v>
+      </c>
+      <c r="D15" s="2">
+        <v>978.25</v>
+      </c>
+      <c r="E15" s="2">
+        <v>-3723.76</v>
+      </c>
+      <c r="G15" s="2">
+        <v>3723.76</v>
+      </c>
+      <c r="I15" s="2">
+        <v>6226.08</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>9</v>
       </c>
       <c r="B16" s="2">
         <v>2702.51</v>
       </c>
-      <c r="J16" s="2">
-        <v>2702.51</v>
-      </c>
-    </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C16" s="2">
+        <v>1125.96</v>
+      </c>
+      <c r="D16" s="2">
+        <v>449.25999999999976</v>
+      </c>
+      <c r="E16" s="2">
+        <v>-2025.81</v>
+      </c>
+      <c r="G16" s="2">
+        <v>2025.81</v>
+      </c>
+      <c r="I16" s="2">
+        <v>3151.77</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>2</v>
       </c>
       <c r="B17" s="2">
         <v>5533.46</v>
       </c>
-      <c r="J17" s="2">
-        <v>5533.46</v>
-      </c>
-    </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C17" s="2">
+        <v>2320.1099999999997</v>
+      </c>
+      <c r="D17" s="2">
+        <v>1066.8900000000003</v>
+      </c>
+      <c r="E17" s="2">
+        <v>-3661.84</v>
+      </c>
+      <c r="G17" s="2">
+        <v>3661.84</v>
+      </c>
+      <c r="I17" s="2">
+        <v>6600.35</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>20</v>
       </c>
       <c r="B18" s="2">
         <v>6747.71</v>
       </c>
-      <c r="J18" s="2">
-        <v>6747.71</v>
-      </c>
-    </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C18" s="2">
+        <v>4603.0600000000004</v>
+      </c>
+      <c r="D18" s="2">
+        <v>3096.6500000000005</v>
+      </c>
+      <c r="E18" s="2">
+        <v>-4657.79</v>
+      </c>
+      <c r="G18" s="2">
+        <v>4657.79</v>
+      </c>
+      <c r="I18" s="2">
+        <v>9844.36</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>19</v>
       </c>
       <c r="B19" s="2">
         <v>4250</v>
       </c>
-      <c r="J19" s="2">
-        <v>4250</v>
-      </c>
-    </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C19" s="2">
+        <v>1753.94</v>
+      </c>
+      <c r="D19" s="2">
+        <v>753.01000000000022</v>
+      </c>
+      <c r="E19" s="2">
+        <v>-2905.89</v>
+      </c>
+      <c r="G19" s="2">
+        <v>2905.89</v>
+      </c>
+      <c r="I19" s="2">
+        <v>5003.01</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>10</v>
       </c>
       <c r="B20" s="2">
         <v>0</v>
       </c>
-      <c r="J20" s="2">
+      <c r="C20" s="2">
+        <v>0</v>
+      </c>
+      <c r="D20" s="2">
+        <v>0</v>
+      </c>
+      <c r="E20" s="2">
+        <v>0</v>
+      </c>
+      <c r="G20" s="2">
+        <v>0</v>
+      </c>
+      <c r="I20" s="2">
         <v>0</v>
       </c>
     </row>
@@ -996,14 +1443,14 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9C8C8C8B-41A6-4BDC-AD33-3B523D6821E6}">
-  <dimension ref="A1:J20"/>
+  <dimension ref="A1:I20"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14.77734375" customWidth="1"/>
-    <col min="2" max="10" width="18.77734375" customWidth="1"/>
+    <col min="2" max="9" width="18.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
@@ -1031,216 +1478,441 @@
       <c r="I1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="J1" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>14</v>
       </c>
       <c r="B2" s="2">
         <v>2800</v>
       </c>
-      <c r="J2" s="2">
-        <v>2800</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C2" s="2">
+        <v>1159.49</v>
+      </c>
+      <c r="D2" s="2">
+        <v>462.09000000000015</v>
+      </c>
+      <c r="E2" s="2">
+        <v>-2000.03</v>
+      </c>
+      <c r="G2" s="2">
+        <v>2000.03</v>
+      </c>
+      <c r="I2" s="2">
+        <v>3262.09</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>16</v>
       </c>
       <c r="B3" s="2">
         <v>3000</v>
       </c>
-      <c r="J3" s="2">
-        <v>3000</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C3" s="2">
+        <v>1069.79</v>
+      </c>
+      <c r="D3" s="2">
+        <v>441.26000000000022</v>
+      </c>
+      <c r="E3" s="2">
+        <v>-2226.5700000000002</v>
+      </c>
+      <c r="G3" s="2">
+        <v>2226.5700000000002</v>
+      </c>
+      <c r="I3" s="2">
+        <v>3441.26</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>11</v>
       </c>
       <c r="B4" s="2">
         <v>1995.96</v>
       </c>
-      <c r="J4" s="2">
-        <v>1995.96</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C4" s="2">
+        <v>883.16000000000008</v>
+      </c>
+      <c r="D4" s="2">
+        <v>356.40999999999985</v>
+      </c>
+      <c r="E4" s="2">
+        <v>-2018.39</v>
+      </c>
+      <c r="G4" s="2">
+        <v>2018.39</v>
+      </c>
+      <c r="I4" s="2">
+        <v>2352.37</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>3</v>
       </c>
       <c r="B5" s="2">
         <v>3395.1</v>
       </c>
-      <c r="J5" s="2">
-        <v>3395.1</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C5" s="2">
+        <v>19264.28</v>
+      </c>
+      <c r="D5" s="2">
+        <v>60695.43</v>
+      </c>
+      <c r="E5" s="2">
+        <v>-44826.25</v>
+      </c>
+      <c r="G5" s="2">
+        <v>44826.25</v>
+      </c>
+      <c r="I5" s="2">
+        <v>64090.53</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>4</v>
       </c>
       <c r="B6" s="2">
         <v>7334.27</v>
       </c>
-      <c r="J6" s="2">
-        <v>7334.27</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C6" s="2">
+        <v>2777.58</v>
+      </c>
+      <c r="D6" s="2">
+        <v>1135.67</v>
+      </c>
+      <c r="E6" s="2">
+        <v>-4571.55</v>
+      </c>
+      <c r="G6" s="2">
+        <v>4571.55</v>
+      </c>
+      <c r="I6" s="2">
+        <v>8469.94</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>13</v>
       </c>
       <c r="B7" s="2">
         <v>3100</v>
       </c>
-      <c r="J7" s="2">
-        <v>3100</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C7" s="2">
+        <v>1105.46</v>
+      </c>
+      <c r="D7" s="2">
+        <v>461.09000000000015</v>
+      </c>
+      <c r="E7" s="2">
+        <v>-2293.21</v>
+      </c>
+      <c r="G7" s="2">
+        <v>2293.21</v>
+      </c>
+      <c r="I7" s="2">
+        <v>3561.09</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>17</v>
       </c>
       <c r="B8" s="2">
         <v>5417</v>
       </c>
-      <c r="J8" s="2">
-        <v>5417</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C8" s="2">
+        <v>3604.8399999999997</v>
+      </c>
+      <c r="D8" s="2">
+        <v>2363.3900000000003</v>
+      </c>
+      <c r="E8" s="2">
+        <v>-4082.75</v>
+      </c>
+      <c r="G8" s="2">
+        <v>4082.75</v>
+      </c>
+      <c r="I8" s="2">
+        <v>7780.39</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>6</v>
       </c>
       <c r="B9" s="2">
         <v>3381</v>
       </c>
-      <c r="J9" s="2">
-        <v>3381</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C9" s="2">
+        <v>1205.6500000000001</v>
+      </c>
+      <c r="D9" s="2">
+        <v>502.15999999999985</v>
+      </c>
+      <c r="E9" s="2">
+        <v>-2555.73</v>
+      </c>
+      <c r="G9" s="2">
+        <v>2555.73</v>
+      </c>
+      <c r="I9" s="2">
+        <v>3883.16</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>15</v>
       </c>
       <c r="B10" s="2">
         <v>3208.4</v>
       </c>
-      <c r="J10" s="2">
-        <v>3208.4</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C10" s="2">
+        <v>1341.24</v>
+      </c>
+      <c r="D10" s="2">
+        <v>563.15000000000009</v>
+      </c>
+      <c r="E10" s="2">
+        <v>-2343.85</v>
+      </c>
+      <c r="G10" s="2">
+        <v>2343.85</v>
+      </c>
+      <c r="I10" s="2">
+        <v>3771.55</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>5</v>
       </c>
       <c r="B11" s="2">
         <v>3286.67</v>
       </c>
-      <c r="J11" s="2">
-        <v>3286.67</v>
-      </c>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C11" s="2">
+        <v>1129.6500000000001</v>
+      </c>
+      <c r="D11" s="2">
+        <v>434.67999999999984</v>
+      </c>
+      <c r="E11" s="2">
+        <v>-2457.5500000000002</v>
+      </c>
+      <c r="G11" s="2">
+        <v>2457.5500000000002</v>
+      </c>
+      <c r="I11" s="2">
+        <v>3721.35</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>7</v>
       </c>
       <c r="B12" s="2">
         <v>3531</v>
       </c>
-      <c r="J12" s="2">
-        <v>3531</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C12" s="2">
+        <v>1259.1399999999999</v>
+      </c>
+      <c r="D12" s="2">
+        <v>529.29</v>
+      </c>
+      <c r="E12" s="2">
+        <v>-2451.39</v>
+      </c>
+      <c r="G12" s="2">
+        <v>2451.39</v>
+      </c>
+      <c r="I12" s="2">
+        <v>4060.29</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>12</v>
       </c>
       <c r="B13" s="2">
         <v>2800</v>
       </c>
-      <c r="J13" s="2">
-        <v>2800</v>
-      </c>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C13" s="2">
+        <v>1159.49</v>
+      </c>
+      <c r="D13" s="2">
+        <v>462.09000000000015</v>
+      </c>
+      <c r="E13" s="2">
+        <v>-1970.4</v>
+      </c>
+      <c r="G13" s="2">
+        <v>1970.4</v>
+      </c>
+      <c r="I13" s="2">
+        <v>3262.09</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>18</v>
       </c>
       <c r="B14" s="2">
         <v>3200</v>
       </c>
-      <c r="J14" s="2">
-        <v>3200</v>
-      </c>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C14" s="2">
+        <v>1141.1199999999999</v>
+      </c>
+      <c r="D14" s="2">
+        <v>478.30000000000018</v>
+      </c>
+      <c r="E14" s="2">
+        <v>-2537.1799999999998</v>
+      </c>
+      <c r="G14" s="2">
+        <v>2537.1799999999998</v>
+      </c>
+      <c r="I14" s="2">
+        <v>3678.3</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>1</v>
       </c>
       <c r="B15" s="2">
         <v>5247.83</v>
       </c>
-      <c r="J15" s="2">
-        <v>5247.83</v>
-      </c>
-    </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C15" s="2">
+        <v>2194.1</v>
+      </c>
+      <c r="D15" s="2">
+        <v>978.25</v>
+      </c>
+      <c r="E15" s="2">
+        <v>-3723.76</v>
+      </c>
+      <c r="G15" s="2">
+        <v>3723.76</v>
+      </c>
+      <c r="I15" s="2">
+        <v>6226.08</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>9</v>
       </c>
       <c r="B16" s="2">
         <v>2700</v>
       </c>
-      <c r="J16" s="2">
-        <v>2700</v>
-      </c>
-    </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C16" s="2">
+        <v>1125.1099999999999</v>
+      </c>
+      <c r="D16" s="2">
+        <v>448.94000000000005</v>
+      </c>
+      <c r="E16" s="2">
+        <v>-2023.83</v>
+      </c>
+      <c r="G16" s="2">
+        <v>2023.83</v>
+      </c>
+      <c r="I16" s="2">
+        <v>3148.94</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>2</v>
       </c>
       <c r="B17" s="2">
         <v>5540.03</v>
       </c>
-      <c r="J17" s="2">
-        <v>5540.03</v>
-      </c>
-    </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C17" s="2">
+        <v>2323.02</v>
+      </c>
+      <c r="D17" s="2">
+        <v>1065.79</v>
+      </c>
+      <c r="E17" s="2">
+        <v>-3663.66</v>
+      </c>
+      <c r="G17" s="2">
+        <v>3663.66</v>
+      </c>
+      <c r="I17" s="2">
+        <v>6605.82</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>20</v>
       </c>
       <c r="B18" s="2">
         <v>4747.71</v>
       </c>
-      <c r="J18" s="2">
-        <v>4747.71</v>
-      </c>
-    </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C18" s="2">
+        <v>3020.5600000000004</v>
+      </c>
+      <c r="D18" s="2">
+        <v>1929.33</v>
+      </c>
+      <c r="E18" s="2">
+        <v>-3245.98</v>
+      </c>
+      <c r="G18" s="2">
+        <v>3245.98</v>
+      </c>
+      <c r="I18" s="2">
+        <v>6677.04</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>19</v>
       </c>
       <c r="B19" s="2">
         <v>4750</v>
       </c>
-      <c r="J19" s="2">
-        <v>4750</v>
-      </c>
-    </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C19" s="2">
+        <v>1974.5100000000002</v>
+      </c>
+      <c r="D19" s="2">
+        <v>867.1899999999996</v>
+      </c>
+      <c r="E19" s="2">
+        <v>-3181.61</v>
+      </c>
+      <c r="G19" s="2">
+        <v>3181.61</v>
+      </c>
+      <c r="I19" s="2">
+        <v>5617.19</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>10</v>
       </c>
       <c r="B20" s="2">
         <v>0</v>
       </c>
-      <c r="J20" s="2">
+      <c r="C20" s="2">
+        <v>0</v>
+      </c>
+      <c r="D20" s="2">
+        <v>0</v>
+      </c>
+      <c r="E20" s="2">
+        <v>0</v>
+      </c>
+      <c r="G20" s="2">
+        <v>0</v>
+      </c>
+      <c r="I20" s="2">
         <v>0</v>
       </c>
     </row>
@@ -1251,14 +1923,14 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{577891D2-093B-4CB8-B5CE-C2FC2771D08B}">
-  <dimension ref="A1:J19"/>
+  <dimension ref="A1:I19"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14.77734375" customWidth="1"/>
-    <col min="2" max="10" width="18.77734375" customWidth="1"/>
+    <col min="2" max="9" width="18.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
@@ -1286,205 +1958,418 @@
       <c r="I1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="J1" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>14</v>
       </c>
       <c r="B2" s="2">
         <v>2800</v>
       </c>
-      <c r="J2" s="2">
-        <v>2800</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C2" s="2">
+        <v>1159.49</v>
+      </c>
+      <c r="D2" s="2">
+        <v>633.34000000000015</v>
+      </c>
+      <c r="E2" s="2">
+        <v>-2071.2800000000002</v>
+      </c>
+      <c r="G2" s="2">
+        <v>2071.2800000000002</v>
+      </c>
+      <c r="I2" s="2">
+        <v>3433.34</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>16</v>
       </c>
       <c r="B3" s="2">
         <v>3000</v>
       </c>
-      <c r="J3" s="2">
-        <v>3000</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C3" s="2">
+        <v>1069.79</v>
+      </c>
+      <c r="D3" s="2">
+        <v>549.05999999999995</v>
+      </c>
+      <c r="E3" s="2">
+        <v>-2234.37</v>
+      </c>
+      <c r="G3" s="2">
+        <v>2234.37</v>
+      </c>
+      <c r="I3" s="2">
+        <v>3549.06</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>11</v>
       </c>
       <c r="B4" s="2">
         <v>2800</v>
       </c>
-      <c r="J4" s="2">
-        <v>2800</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C4" s="2">
+        <v>1159.49</v>
+      </c>
+      <c r="D4" s="2">
+        <v>562.09000000000015</v>
+      </c>
+      <c r="E4" s="2">
+        <v>-2018.26</v>
+      </c>
+      <c r="G4" s="2">
+        <v>2018.26</v>
+      </c>
+      <c r="I4" s="2">
+        <v>3362.09</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>4</v>
       </c>
       <c r="B5" s="2">
         <v>7250</v>
       </c>
-      <c r="J5" s="2">
-        <v>7250</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C5" s="2">
+        <v>2769.22</v>
+      </c>
+      <c r="D5" s="2">
+        <v>1242.9599999999991</v>
+      </c>
+      <c r="E5" s="2">
+        <v>-4517.68</v>
+      </c>
+      <c r="G5" s="2">
+        <v>4517.68</v>
+      </c>
+      <c r="I5" s="2">
+        <v>8492.9599999999991</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>13</v>
       </c>
       <c r="B6" s="2">
         <v>3100</v>
       </c>
-      <c r="J6" s="2">
-        <v>3100</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C6" s="2">
+        <v>1105.46</v>
+      </c>
+      <c r="D6" s="2">
+        <v>566.29</v>
+      </c>
+      <c r="E6" s="2">
+        <v>-2298.41</v>
+      </c>
+      <c r="G6" s="2">
+        <v>2298.41</v>
+      </c>
+      <c r="I6" s="2">
+        <v>3666.29</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>17</v>
       </c>
       <c r="B7" s="2">
         <v>5417</v>
       </c>
-      <c r="J7" s="2">
-        <v>5417</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C7" s="2">
+        <v>3604.8399999999997</v>
+      </c>
+      <c r="D7" s="2">
+        <v>2468.59</v>
+      </c>
+      <c r="E7" s="2">
+        <v>-4087.95</v>
+      </c>
+      <c r="G7" s="2">
+        <v>4087.95</v>
+      </c>
+      <c r="I7" s="2">
+        <v>7885.59</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>6</v>
       </c>
       <c r="B8" s="2">
         <v>3381</v>
       </c>
-      <c r="J8" s="2">
-        <v>3381</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C8" s="2">
+        <v>1205.6500000000001</v>
+      </c>
+      <c r="D8" s="2">
+        <v>615.15999999999985</v>
+      </c>
+      <c r="E8" s="2">
+        <v>-2568.73</v>
+      </c>
+      <c r="G8" s="2">
+        <v>2568.73</v>
+      </c>
+      <c r="I8" s="2">
+        <v>3996.16</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>15</v>
       </c>
       <c r="B9" s="2">
         <v>3203.15</v>
       </c>
-      <c r="J9" s="2">
-        <v>3203.15</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C9" s="2">
+        <v>1339.3600000000001</v>
+      </c>
+      <c r="D9" s="2">
+        <v>662.36999999999989</v>
+      </c>
+      <c r="E9" s="2">
+        <v>-2339.84</v>
+      </c>
+      <c r="G9" s="2">
+        <v>2339.84</v>
+      </c>
+      <c r="I9" s="2">
+        <v>3865.52</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>5</v>
       </c>
       <c r="B10" s="2">
         <v>3286.67</v>
       </c>
-      <c r="J10" s="2">
-        <v>3286.67</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C10" s="2">
+        <v>1129.6500000000001</v>
+      </c>
+      <c r="D10" s="2">
+        <v>532.07999999999993</v>
+      </c>
+      <c r="E10" s="2">
+        <v>-2454.9499999999998</v>
+      </c>
+      <c r="G10" s="2">
+        <v>2454.9499999999998</v>
+      </c>
+      <c r="I10" s="2">
+        <v>3818.75</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>7</v>
       </c>
       <c r="B11" s="2">
         <v>3531</v>
       </c>
-      <c r="J11" s="2">
-        <v>3531</v>
-      </c>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C11" s="2">
+        <v>1259.1399999999999</v>
+      </c>
+      <c r="D11" s="2">
+        <v>650.35999999999967</v>
+      </c>
+      <c r="E11" s="2">
+        <v>-2472.46</v>
+      </c>
+      <c r="G11" s="2">
+        <v>2472.46</v>
+      </c>
+      <c r="I11" s="2">
+        <v>4181.3599999999997</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>12</v>
       </c>
       <c r="B12" s="2">
         <v>2800</v>
       </c>
-      <c r="J12" s="2">
-        <v>2800</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C12" s="2">
+        <v>1159.49</v>
+      </c>
+      <c r="D12" s="2">
+        <v>562.09000000000015</v>
+      </c>
+      <c r="E12" s="2">
+        <v>-1970.4</v>
+      </c>
+      <c r="G12" s="2">
+        <v>1970.4</v>
+      </c>
+      <c r="I12" s="2">
+        <v>3362.09</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>18</v>
       </c>
       <c r="B13" s="2">
         <v>3200</v>
       </c>
-      <c r="J13" s="2">
-        <v>3200</v>
-      </c>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C13" s="2">
+        <v>1141.1199999999999</v>
+      </c>
+      <c r="D13" s="2">
+        <v>580.90000000000009</v>
+      </c>
+      <c r="E13" s="2">
+        <v>-2539.7800000000002</v>
+      </c>
+      <c r="G13" s="2">
+        <v>2539.7800000000002</v>
+      </c>
+      <c r="I13" s="2">
+        <v>3780.9</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>1</v>
       </c>
       <c r="B14" s="2">
         <v>5247.83</v>
       </c>
-      <c r="J14" s="2">
-        <v>5247.83</v>
-      </c>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C14" s="2">
+        <v>2194.1</v>
+      </c>
+      <c r="D14" s="2">
+        <v>1088.6499999999996</v>
+      </c>
+      <c r="E14" s="2">
+        <v>-3734.16</v>
+      </c>
+      <c r="G14" s="2">
+        <v>3734.16</v>
+      </c>
+      <c r="I14" s="2">
+        <v>6336.48</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>9</v>
       </c>
       <c r="B15" s="2">
         <v>2575.39</v>
       </c>
-      <c r="J15" s="2">
-        <v>2575.39</v>
-      </c>
-    </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C15" s="2">
+        <v>1082.28</v>
+      </c>
+      <c r="D15" s="2">
+        <v>532.55999999999995</v>
+      </c>
+      <c r="E15" s="2">
+        <v>-1925.67</v>
+      </c>
+      <c r="G15" s="2">
+        <v>1925.67</v>
+      </c>
+      <c r="I15" s="2">
+        <v>3107.95</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>2</v>
       </c>
       <c r="B16" s="2">
         <v>5474.36</v>
       </c>
-      <c r="J16" s="2">
-        <v>5474.36</v>
-      </c>
-    </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C16" s="2">
+        <v>2294.02</v>
+      </c>
+      <c r="D16" s="2">
+        <v>1174.1800000000003</v>
+      </c>
+      <c r="E16" s="2">
+        <v>-3642.72</v>
+      </c>
+      <c r="G16" s="2">
+        <v>3642.72</v>
+      </c>
+      <c r="I16" s="2">
+        <v>6648.54</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>20</v>
       </c>
       <c r="B17" s="2">
         <v>4747.71</v>
       </c>
-      <c r="J17" s="2">
-        <v>4747.71</v>
-      </c>
-    </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C17" s="2">
+        <v>3185.95</v>
+      </c>
+      <c r="D17" s="2">
+        <v>2210.3199999999997</v>
+      </c>
+      <c r="E17" s="2">
+        <v>-3261.58</v>
+      </c>
+      <c r="G17" s="2">
+        <v>3261.58</v>
+      </c>
+      <c r="I17" s="2">
+        <v>6958.03</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>19</v>
       </c>
       <c r="B18" s="2">
         <v>4250</v>
       </c>
-      <c r="J18" s="2">
-        <v>4250</v>
-      </c>
-    </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C18" s="2">
+        <v>1753.94</v>
+      </c>
+      <c r="D18" s="2">
+        <v>860.8100000000004</v>
+      </c>
+      <c r="E18" s="2">
+        <v>-2913.69</v>
+      </c>
+      <c r="G18" s="2">
+        <v>2913.69</v>
+      </c>
+      <c r="I18" s="2">
+        <v>5110.8100000000004</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>10</v>
       </c>
       <c r="B19" s="2">
         <v>0</v>
       </c>
-      <c r="J19" s="2">
+      <c r="C19" s="2">
+        <v>0</v>
+      </c>
+      <c r="D19" s="2">
+        <v>0</v>
+      </c>
+      <c r="E19" s="2">
+        <v>0</v>
+      </c>
+      <c r="G19" s="2">
+        <v>0</v>
+      </c>
+      <c r="I19" s="2">
         <v>0</v>
       </c>
     </row>
@@ -1495,14 +2380,14 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CA707A39-B264-4FEF-B150-828888115482}">
-  <dimension ref="A1:J19"/>
+  <dimension ref="A1:I19"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14.77734375" customWidth="1"/>
-    <col min="2" max="10" width="18.77734375" customWidth="1"/>
+    <col min="2" max="9" width="18.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
@@ -1530,205 +2415,418 @@
       <c r="I1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="J1" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>14</v>
       </c>
       <c r="B2" s="2">
         <v>2900</v>
       </c>
-      <c r="J2" s="2">
-        <v>2900</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C2" s="2">
+        <v>1193.8499999999999</v>
+      </c>
+      <c r="D2" s="2">
+        <v>475.23</v>
+      </c>
+      <c r="E2" s="2">
+        <v>-2075.13</v>
+      </c>
+      <c r="G2" s="2">
+        <v>2075.13</v>
+      </c>
+      <c r="I2" s="2">
+        <v>3375.23</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>16</v>
       </c>
       <c r="B3" s="2">
         <v>3000</v>
       </c>
-      <c r="J3" s="2">
-        <v>3000</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C3" s="2">
+        <v>1069.79</v>
+      </c>
+      <c r="D3" s="2">
+        <v>449.05999999999995</v>
+      </c>
+      <c r="E3" s="2">
+        <v>-2278.58</v>
+      </c>
+      <c r="G3" s="2">
+        <v>2278.58</v>
+      </c>
+      <c r="I3" s="2">
+        <v>3449.06</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>11</v>
       </c>
       <c r="B4" s="2">
         <v>2800</v>
       </c>
-      <c r="J4" s="2">
-        <v>2800</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C4" s="2">
+        <v>1159.49</v>
+      </c>
+      <c r="D4" s="2">
+        <v>462.09000000000015</v>
+      </c>
+      <c r="E4" s="2">
+        <v>-2002.31</v>
+      </c>
+      <c r="G4" s="2">
+        <v>2002.31</v>
+      </c>
+      <c r="I4" s="2">
+        <v>3262.09</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>4</v>
       </c>
       <c r="B5" s="2">
         <v>7250</v>
       </c>
-      <c r="J5" s="2">
-        <v>7250</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C5" s="2">
+        <v>2769.25</v>
+      </c>
+      <c r="D5" s="2">
+        <v>1142.9699999999993</v>
+      </c>
+      <c r="E5" s="2">
+        <v>-4494</v>
+      </c>
+      <c r="G5" s="2">
+        <v>4494</v>
+      </c>
+      <c r="I5" s="2">
+        <v>8392.9699999999993</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>13</v>
       </c>
       <c r="B6" s="2">
         <v>3700</v>
       </c>
-      <c r="J6" s="2">
-        <v>3700</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C6" s="2">
+        <v>1319.4099999999999</v>
+      </c>
+      <c r="D6" s="2">
+        <v>548.8100000000004</v>
+      </c>
+      <c r="E6" s="2">
+        <v>-2765.84</v>
+      </c>
+      <c r="G6" s="2">
+        <v>2765.84</v>
+      </c>
+      <c r="I6" s="2">
+        <v>4248.8100000000004</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>17</v>
       </c>
       <c r="B7" s="2">
         <v>5417</v>
       </c>
-      <c r="J7" s="2">
-        <v>5417</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C7" s="2">
+        <v>3604.8399999999997</v>
+      </c>
+      <c r="D7" s="2">
+        <v>2376.3900000000003</v>
+      </c>
+      <c r="E7" s="2">
+        <v>-4188.55</v>
+      </c>
+      <c r="G7" s="2">
+        <v>4188.55</v>
+      </c>
+      <c r="I7" s="2">
+        <v>7793.39</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>6</v>
       </c>
       <c r="B8" s="2">
         <v>3381</v>
       </c>
-      <c r="J8" s="2">
-        <v>3381</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C8" s="2">
+        <v>1205.6500000000001</v>
+      </c>
+      <c r="D8" s="2">
+        <v>517.76000000000022</v>
+      </c>
+      <c r="E8" s="2">
+        <v>-2593.4699999999998</v>
+      </c>
+      <c r="G8" s="2">
+        <v>2593.4699999999998</v>
+      </c>
+      <c r="I8" s="2">
+        <v>3898.76</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>15</v>
       </c>
       <c r="B9" s="2">
         <v>3200</v>
       </c>
-      <c r="J9" s="2">
-        <v>3200</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C9" s="2">
+        <v>1338.23</v>
+      </c>
+      <c r="D9" s="2">
+        <v>561.90000000000009</v>
+      </c>
+      <c r="E9" s="2">
+        <v>-2332.21</v>
+      </c>
+      <c r="G9" s="2">
+        <v>2332.21</v>
+      </c>
+      <c r="I9" s="2">
+        <v>3761.9</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>5</v>
       </c>
       <c r="B10" s="2">
         <v>3451</v>
       </c>
-      <c r="J10" s="2">
-        <v>3451</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C10" s="2">
+        <v>1230.6199999999999</v>
+      </c>
+      <c r="D10" s="2">
+        <v>504.59999999999991</v>
+      </c>
+      <c r="E10" s="2">
+        <v>-2597.85</v>
+      </c>
+      <c r="G10" s="2">
+        <v>2597.85</v>
+      </c>
+      <c r="I10" s="2">
+        <v>3955.6</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>7</v>
       </c>
       <c r="B11" s="2">
         <v>3531</v>
       </c>
-      <c r="J11" s="2">
-        <v>3531</v>
-      </c>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C11" s="2">
+        <v>1259.1399999999999</v>
+      </c>
+      <c r="D11" s="2">
+        <v>531.88999999999987</v>
+      </c>
+      <c r="E11" s="2">
+        <v>-2459.77</v>
+      </c>
+      <c r="G11" s="2">
+        <v>2459.77</v>
+      </c>
+      <c r="I11" s="2">
+        <v>4062.89</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>12</v>
       </c>
       <c r="B12" s="2">
         <v>2900</v>
       </c>
-      <c r="J12" s="2">
-        <v>2900</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C12" s="2">
+        <v>1193.8499999999999</v>
+      </c>
+      <c r="D12" s="2">
+        <v>475.23</v>
+      </c>
+      <c r="E12" s="2">
+        <v>-2044.44</v>
+      </c>
+      <c r="G12" s="2">
+        <v>2044.44</v>
+      </c>
+      <c r="I12" s="2">
+        <v>3375.23</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>18</v>
       </c>
       <c r="B13" s="2">
         <v>3200</v>
       </c>
-      <c r="J13" s="2">
-        <v>3200</v>
-      </c>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C13" s="2">
+        <v>1141.1199999999999</v>
+      </c>
+      <c r="D13" s="2">
+        <v>475.69999999999982</v>
+      </c>
+      <c r="E13" s="2">
+        <v>-2476.9499999999998</v>
+      </c>
+      <c r="G13" s="2">
+        <v>2476.9499999999998</v>
+      </c>
+      <c r="I13" s="2">
+        <v>3675.7</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>1</v>
       </c>
       <c r="B14" s="2">
         <v>5247.83</v>
       </c>
-      <c r="J14" s="2">
-        <v>5247.83</v>
-      </c>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C14" s="2">
+        <v>2194.1</v>
+      </c>
+      <c r="D14" s="2">
+        <v>980.85000000000036</v>
+      </c>
+      <c r="E14" s="2">
+        <v>-4034.58</v>
+      </c>
+      <c r="G14" s="2">
+        <v>4034.58</v>
+      </c>
+      <c r="I14" s="2">
+        <v>6228.68</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>9</v>
       </c>
       <c r="B15" s="2">
         <v>2800</v>
       </c>
-      <c r="J15" s="2">
-        <v>2800</v>
-      </c>
-    </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C15" s="2">
+        <v>1159.49</v>
+      </c>
+      <c r="D15" s="2">
+        <v>462.09000000000015</v>
+      </c>
+      <c r="E15" s="2">
+        <v>-2102.6</v>
+      </c>
+      <c r="G15" s="2">
+        <v>2102.6</v>
+      </c>
+      <c r="I15" s="2">
+        <v>3262.09</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>2</v>
       </c>
       <c r="B16" s="2">
         <v>5474.36</v>
       </c>
-      <c r="J16" s="2">
-        <v>5474.36</v>
-      </c>
-    </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C16" s="2">
+        <v>2294.02</v>
+      </c>
+      <c r="D16" s="2">
+        <v>1074.1800000000003</v>
+      </c>
+      <c r="E16" s="2">
+        <v>-3656.12</v>
+      </c>
+      <c r="G16" s="2">
+        <v>3656.12</v>
+      </c>
+      <c r="I16" s="2">
+        <v>6548.54</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>20</v>
       </c>
       <c r="B17" s="2">
         <v>4747.71</v>
       </c>
-      <c r="J17" s="2">
-        <v>4747.71</v>
-      </c>
-    </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C17" s="2">
+        <v>3185.95</v>
+      </c>
+      <c r="D17" s="2">
+        <v>2107.7200000000003</v>
+      </c>
+      <c r="E17" s="2">
+        <v>-3394.52</v>
+      </c>
+      <c r="G17" s="2">
+        <v>3394.52</v>
+      </c>
+      <c r="I17" s="2">
+        <v>6855.43</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>19</v>
       </c>
       <c r="B18" s="2">
         <v>4250</v>
       </c>
-      <c r="J18" s="2">
-        <v>4250</v>
-      </c>
-    </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C18" s="2">
+        <v>1753.94</v>
+      </c>
+      <c r="D18" s="2">
+        <v>758.21</v>
+      </c>
+      <c r="E18" s="2">
+        <v>-2911.09</v>
+      </c>
+      <c r="G18" s="2">
+        <v>2911.09</v>
+      </c>
+      <c r="I18" s="2">
+        <v>5008.21</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>10</v>
       </c>
       <c r="B19" s="2">
         <v>0</v>
       </c>
-      <c r="J19" s="2">
+      <c r="C19" s="2">
+        <v>0</v>
+      </c>
+      <c r="D19" s="2">
+        <v>0</v>
+      </c>
+      <c r="E19" s="2">
+        <v>0</v>
+      </c>
+      <c r="G19" s="2">
+        <v>0</v>
+      </c>
+      <c r="I19" s="2">
         <v>0</v>
       </c>
     </row>
@@ -1739,14 +2837,14 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{25107736-CA63-405D-9FDF-3F7D8EF9ED6E}">
-  <dimension ref="A1:J19"/>
+  <dimension ref="A1:I19"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14.77734375" customWidth="1"/>
-    <col min="2" max="10" width="18.77734375" customWidth="1"/>
+    <col min="2" max="9" width="18.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
@@ -1774,205 +2872,418 @@
       <c r="I1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="J1" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>14</v>
       </c>
       <c r="B2" s="2">
         <v>2900.57</v>
       </c>
-      <c r="J2" s="2">
-        <v>2900.57</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C2" s="2">
+        <v>1194.03</v>
+      </c>
+      <c r="D2" s="2">
+        <v>1475.2999999999997</v>
+      </c>
+      <c r="E2" s="2">
+        <v>-3075.57</v>
+      </c>
+      <c r="G2" s="2">
+        <v>3075.57</v>
+      </c>
+      <c r="I2" s="2">
+        <v>4375.87</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>16</v>
       </c>
       <c r="B3" s="2">
         <v>3000</v>
       </c>
-      <c r="J3" s="2">
-        <v>3000</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C3" s="2">
+        <v>1069.79</v>
+      </c>
+      <c r="D3" s="2">
+        <v>1449.0600000000004</v>
+      </c>
+      <c r="E3" s="2">
+        <v>-3278.58</v>
+      </c>
+      <c r="G3" s="2">
+        <v>3278.58</v>
+      </c>
+      <c r="I3" s="2">
+        <v>4449.0600000000004</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>11</v>
       </c>
       <c r="B4" s="2">
         <v>2800</v>
       </c>
-      <c r="J4" s="2">
-        <v>2800</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C4" s="2">
+        <v>1159.49</v>
+      </c>
+      <c r="D4" s="2">
+        <v>1462.0900000000001</v>
+      </c>
+      <c r="E4" s="2">
+        <v>-3002.31</v>
+      </c>
+      <c r="G4" s="2">
+        <v>3002.31</v>
+      </c>
+      <c r="I4" s="2">
+        <v>4262.09</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>4</v>
       </c>
       <c r="B5" s="2">
         <v>7250</v>
       </c>
-      <c r="J5" s="2">
-        <v>7250</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C5" s="2">
+        <v>2864.56</v>
+      </c>
+      <c r="D5" s="2">
+        <v>2150.7700000000004</v>
+      </c>
+      <c r="E5" s="2">
+        <v>-5228.25</v>
+      </c>
+      <c r="G5" s="2">
+        <v>5228.25</v>
+      </c>
+      <c r="I5" s="2">
+        <v>9400.77</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>13</v>
       </c>
       <c r="B6" s="2">
         <v>3200</v>
       </c>
-      <c r="J6" s="2">
-        <v>3200</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C6" s="2">
+        <v>1141.1199999999999</v>
+      </c>
+      <c r="D6" s="2">
+        <v>1473.1000000000004</v>
+      </c>
+      <c r="E6" s="2">
+        <v>-3390.52</v>
+      </c>
+      <c r="G6" s="2">
+        <v>3390.52</v>
+      </c>
+      <c r="I6" s="2">
+        <v>4673.1000000000004</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>17</v>
       </c>
       <c r="B7" s="2">
         <v>5417</v>
       </c>
-      <c r="J7" s="2">
-        <v>5417</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C7" s="2">
+        <v>3700.14</v>
+      </c>
+      <c r="D7" s="2">
+        <v>3373.7900000000009</v>
+      </c>
+      <c r="E7" s="2">
+        <v>-5090.6499999999996</v>
+      </c>
+      <c r="G7" s="2">
+        <v>5090.6499999999996</v>
+      </c>
+      <c r="I7" s="2">
+        <v>8790.7900000000009</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>6</v>
       </c>
       <c r="B8" s="2">
         <v>3381</v>
       </c>
-      <c r="J8" s="2">
-        <v>3381</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C8" s="2">
+        <v>1205.6500000000001</v>
+      </c>
+      <c r="D8" s="2">
+        <v>1504.7600000000002</v>
+      </c>
+      <c r="E8" s="2">
+        <v>-3580.47</v>
+      </c>
+      <c r="G8" s="2">
+        <v>3580.47</v>
+      </c>
+      <c r="I8" s="2">
+        <v>4885.76</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>15</v>
       </c>
       <c r="B9" s="2">
         <v>3200</v>
       </c>
-      <c r="J9" s="2">
-        <v>3200</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C9" s="2">
+        <v>1338.23</v>
+      </c>
+      <c r="D9" s="2">
+        <v>1564.5</v>
+      </c>
+      <c r="E9" s="2">
+        <v>-3334.81</v>
+      </c>
+      <c r="G9" s="2">
+        <v>3334.81</v>
+      </c>
+      <c r="I9" s="2">
+        <v>4764.5</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>5</v>
       </c>
       <c r="B10" s="2">
         <v>3451</v>
       </c>
-      <c r="J10" s="2">
-        <v>3451</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C10" s="2">
+        <v>1230.6199999999999</v>
+      </c>
+      <c r="D10" s="2">
+        <v>1504.6000000000004</v>
+      </c>
+      <c r="E10" s="2">
+        <v>-3597.85</v>
+      </c>
+      <c r="G10" s="2">
+        <v>3597.85</v>
+      </c>
+      <c r="I10" s="2">
+        <v>4955.6000000000004</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>7</v>
       </c>
       <c r="B11" s="2">
         <v>3531</v>
       </c>
-      <c r="J11" s="2">
-        <v>3531</v>
-      </c>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C11" s="2">
+        <v>1259.1399999999999</v>
+      </c>
+      <c r="D11" s="2">
+        <v>1541.0900000000001</v>
+      </c>
+      <c r="E11" s="2">
+        <v>-3468.97</v>
+      </c>
+      <c r="G11" s="2">
+        <v>3468.97</v>
+      </c>
+      <c r="I11" s="2">
+        <v>5072.09</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>12</v>
       </c>
       <c r="B12" s="2">
         <v>2900</v>
       </c>
-      <c r="J12" s="2">
-        <v>2900</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C12" s="2">
+        <v>1193.8499999999999</v>
+      </c>
+      <c r="D12" s="2">
+        <v>1475.2299999999996</v>
+      </c>
+      <c r="E12" s="2">
+        <v>-3044.44</v>
+      </c>
+      <c r="G12" s="2">
+        <v>3044.44</v>
+      </c>
+      <c r="I12" s="2">
+        <v>4375.2299999999996</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>18</v>
       </c>
       <c r="B13" s="2">
         <v>3200</v>
       </c>
-      <c r="J13" s="2">
-        <v>3200</v>
-      </c>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C13" s="2">
+        <v>1141.1199999999999</v>
+      </c>
+      <c r="D13" s="2">
+        <v>1478.3000000000002</v>
+      </c>
+      <c r="E13" s="2">
+        <v>-3479.55</v>
+      </c>
+      <c r="G13" s="2">
+        <v>3479.55</v>
+      </c>
+      <c r="I13" s="2">
+        <v>4678.3</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>1</v>
       </c>
       <c r="B14" s="2">
         <v>5247.83</v>
       </c>
-      <c r="J14" s="2">
-        <v>5247.83</v>
-      </c>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C14" s="2">
+        <v>2194.1</v>
+      </c>
+      <c r="D14" s="2">
+        <v>1983.4499999999998</v>
+      </c>
+      <c r="E14" s="2">
+        <v>-5037.18</v>
+      </c>
+      <c r="G14" s="2">
+        <v>5037.18</v>
+      </c>
+      <c r="I14" s="2">
+        <v>7231.28</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>9</v>
       </c>
       <c r="B15" s="2">
         <v>2800</v>
       </c>
-      <c r="J15" s="2">
-        <v>2800</v>
-      </c>
-    </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C15" s="2">
+        <v>1159.49</v>
+      </c>
+      <c r="D15" s="2">
+        <v>1462.0900000000001</v>
+      </c>
+      <c r="E15" s="2">
+        <v>-3102.6</v>
+      </c>
+      <c r="G15" s="2">
+        <v>3102.6</v>
+      </c>
+      <c r="I15" s="2">
+        <v>4262.09</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>2</v>
       </c>
       <c r="B16" s="2">
         <v>4687.9799999999996</v>
       </c>
-      <c r="J16" s="2">
-        <v>4687.9799999999996</v>
-      </c>
-    </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C16" s="2">
+        <v>2042.4099999999999</v>
+      </c>
+      <c r="D16" s="2">
+        <v>1860.7900000000009</v>
+      </c>
+      <c r="E16" s="2">
+        <v>-4402.4399999999996</v>
+      </c>
+      <c r="G16" s="2">
+        <v>4402.4399999999996</v>
+      </c>
+      <c r="I16" s="2">
+        <v>6548.77</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>20</v>
       </c>
       <c r="B17" s="2">
         <v>9747.7099999999991</v>
       </c>
-      <c r="J17" s="2">
-        <v>9747.7099999999991</v>
-      </c>
-    </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C17" s="2">
+        <v>7007.76</v>
+      </c>
+      <c r="D17" s="2">
+        <v>5770.2900000000009</v>
+      </c>
+      <c r="E17" s="2">
+        <v>-7879.31</v>
+      </c>
+      <c r="G17" s="2">
+        <v>7879.31</v>
+      </c>
+      <c r="I17" s="2">
+        <v>15518</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>19</v>
       </c>
       <c r="B18" s="2">
         <v>4250</v>
       </c>
-      <c r="J18" s="2">
-        <v>4250</v>
-      </c>
-    </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C18" s="2">
+        <v>1753.94</v>
+      </c>
+      <c r="D18" s="2">
+        <v>1760.8100000000004</v>
+      </c>
+      <c r="E18" s="2">
+        <v>-3913.69</v>
+      </c>
+      <c r="G18" s="2">
+        <v>3913.69</v>
+      </c>
+      <c r="I18" s="2">
+        <v>6010.81</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>10</v>
       </c>
       <c r="B19" s="2">
         <v>0</v>
       </c>
-      <c r="J19" s="2">
+      <c r="C19" s="2">
+        <v>0</v>
+      </c>
+      <c r="D19" s="2">
+        <v>0</v>
+      </c>
+      <c r="E19" s="2">
+        <v>0</v>
+      </c>
+      <c r="G19" s="2">
+        <v>0</v>
+      </c>
+      <c r="I19" s="2">
         <v>0</v>
       </c>
     </row>

</xml_diff>